<commit_message>
Fix typo in pinmap file
</commit_message>
<xml_diff>
--- a/STM pinmap.xlsx
+++ b/STM pinmap.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Имя</t>
   </si>
@@ -169,6 +169,9 @@
   </si>
   <si>
     <t>TIM3_CH2, I2C1_SMBA, SPI1_MOSI, SPI3_MOSI/I2S3_SD, CAN2_RX, OTG_HS_ULPI_D7, ETH_PPS_OUT, FMC_SDCKE1, DCMI_D10, EVENTOUT</t>
+  </si>
+  <si>
+    <t>R_A_VN</t>
   </si>
 </sst>
 </file>
@@ -680,7 +683,7 @@
         <v>19</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
add info about additional pins (extension board)
</commit_message>
<xml_diff>
--- a/STM pinmap.xlsx
+++ b/STM pinmap.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
   <si>
     <t>Имя</t>
   </si>
@@ -24,9 +24,6 @@
     <t>Назначение</t>
   </si>
   <si>
-    <t>Функции</t>
-  </si>
-  <si>
     <t>PG1</t>
   </si>
   <si>
@@ -172,18 +169,99 @@
   </si>
   <si>
     <t>R_A_VN</t>
+  </si>
+  <si>
+    <t>PD5</t>
+  </si>
+  <si>
+    <t>USART2_TX</t>
+  </si>
+  <si>
+    <t>USART2_TX, FMC_NWE, EVENTOUT</t>
+  </si>
+  <si>
+    <t>I2C2_SDA, FMC_A0, EVENTOUT</t>
+  </si>
+  <si>
+    <t>I2C2_SDA</t>
+  </si>
+  <si>
+    <t>PF0</t>
+  </si>
+  <si>
+    <t>PF1</t>
+  </si>
+  <si>
+    <t>I2C2_SCL</t>
+  </si>
+  <si>
+    <t>I2C2_SCL, FMC_A1, EVENTOUT</t>
+  </si>
+  <si>
+    <t>Управление состоянием реле</t>
+  </si>
+  <si>
+    <t>Все альтернативные функции</t>
+  </si>
+  <si>
+    <r>
+      <t>Подключение LCD 1602 (I</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C: PCF8574T)</t>
+    </r>
+  </si>
+  <si>
+    <t>Вывод отладочной информации</t>
+  </si>
+  <si>
+    <t>PF2</t>
+  </si>
+  <si>
+    <t>I2C2_SMBA, FMC_A2, EVENTOUT</t>
+  </si>
+  <si>
+    <t>Считывание состояния кнопки (input pull-up)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -228,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -238,6 +316,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -540,255 +633,348 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="124.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>88</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>87</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>116</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>113</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="E9" s="6"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>112</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="E10" s="6"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>111</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>99</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="E12" s="6"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>98</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="D14" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="E14" s="6"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>47</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="D15" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="E15" s="6"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>133</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="E16" s="6"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>135</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="D17" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>10</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>11</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>12</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>119</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E17"/>
+    <mergeCell ref="E18:E19"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update pinout for ext board
</commit_message>
<xml_diff>
--- a/STM pinmap.xlsx
+++ b/STM pinmap.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
   <si>
     <t>Имя</t>
   </si>
@@ -153,51 +153,15 @@
     <t>TIM3_CH3, TIM8_CH3, USART6_CK, SDIO_D0, DCMI_D2, EVENTOUT</t>
   </si>
   <si>
-    <t>SPI2_MISO, I2S2ext_SD, OTG_HS_ULPI_DIR, ETH_MII_TXD2, FMC_SDNE0, EVENTOUT, ADC123_IN12</t>
-  </si>
-  <si>
-    <t>TIM1_CH3N, TIM3_CH4, TIM8_CH3N, LCD_R6, OTG_HS_ULPI_D2, ETH_MII_RXD3, EVENTOUT, ADC12_IN9</t>
-  </si>
-  <si>
     <t>JTDO/TRACESWO, TIM2_CH2, SPI1_SCK, SPI3_SCK/I2S3_CK, EVENTOUT</t>
   </si>
   <si>
     <t>Номер вывода (LQFP144)</t>
   </si>
   <si>
-    <t>TIM3_CH2, I2C1_SMBA, SPI1_MOSI, SPI3_MOSI/I2S3_SD, CAN2_RX, OTG_HS_ULPI_D7, ETH_PPS_OUT, FMC_SDCKE1, DCMI_D10, EVENTOUT</t>
-  </si>
-  <si>
     <t>R_A_VN</t>
   </si>
   <si>
-    <t>PD5</t>
-  </si>
-  <si>
-    <t>USART2_TX</t>
-  </si>
-  <si>
-    <t>USART2_TX, FMC_NWE, EVENTOUT</t>
-  </si>
-  <si>
-    <t>I2C2_SDA, FMC_A0, EVENTOUT</t>
-  </si>
-  <si>
-    <t>I2C2_SDA</t>
-  </si>
-  <si>
-    <t>PF0</t>
-  </si>
-  <si>
-    <t>PF1</t>
-  </si>
-  <si>
-    <t>I2C2_SCL</t>
-  </si>
-  <si>
-    <t>I2C2_SCL, FMC_A1, EVENTOUT</t>
-  </si>
-  <si>
     <t>Управление состоянием реле</t>
   </si>
   <si>
@@ -234,25 +198,308 @@
     <t>Вывод отладочной информации</t>
   </si>
   <si>
-    <t>PF2</t>
-  </si>
-  <si>
-    <t>I2C2_SMBA, FMC_A2, EVENTOUT</t>
-  </si>
-  <si>
     <t>Считывание состояния кнопки (input pull-up)</t>
+  </si>
+  <si>
+    <t>PB8</t>
+  </si>
+  <si>
+    <t>I2C1_SCL</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">TIM3_CH2, I2C1_SMBA, SPI1_MOSI, SPI3_MOSI/I2S3_SD, CAN2_RX, OTG_HS_ULPI_D7, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ETH_PPS_OUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, FMC_SDCKE1, DCMI_D10, EVENTOUT</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">TIM1_CH3N, TIM3_CH4, TIM8_CH3N, LCD_R6, OTG_HS_ULPI_D2, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ETH_MII_RXD3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, EVENTOUT, ADC12_IN9</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SPI2_MISO, I2S2ext_SD, OTG_HS_ULPI_DIR, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ETH_MII_TXD2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, FMC_SDNE0, EVENTOUT, ADC123_IN12</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">TIM4_CH3, TIM10_CH1, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I2C1_SCL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, CAN1_RX, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ETH_MII_TXD3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, SDIO_D4, DCMI_D6, LCD_B6, EVENTOUT</t>
+    </r>
+  </si>
+  <si>
+    <t>PB9</t>
+  </si>
+  <si>
+    <t>I2C1_SDA</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">TIM4_CH4, TIM11_CH1, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I2C1_SDA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, SPI2_NSS/I2S2_WS, CAN1_TX, SDIO_D5, DCMI_D7, LCD_B7, EVENTOUT</t>
+    </r>
+  </si>
+  <si>
+    <t>PG14</t>
+  </si>
+  <si>
+    <t>PG9</t>
+  </si>
+  <si>
+    <t>USART6_TX</t>
+  </si>
+  <si>
+    <t>USART6_RX</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>USART6_RX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, FMC_NE2/FMC_NCE3, DCMI_VSYNC(9), EVENTOUT</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SPI6_MOSI, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>USART6_TX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ETH_MII_TXD1/ETH_ RMII_TXD1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, FMC_A25, EVENTOUT</t>
+    </r>
+  </si>
+  <si>
+    <t>Плата</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>ext</t>
+  </si>
+  <si>
+    <t>PC0</t>
+  </si>
+  <si>
+    <t>OTG_HS_ULPI_STP, FMC_SDNWE, ADC123_IN10, EVENTOUT</t>
+  </si>
+  <si>
+    <t>INPUT_LEFT</t>
+  </si>
+  <si>
+    <t>INPUT_MID</t>
+  </si>
+  <si>
+    <t>INPUT_RIGHT</t>
+  </si>
+  <si>
+    <t>PF3</t>
+  </si>
+  <si>
+    <t>FMC_A3, EVENTOUT, ADC3_IN9</t>
+  </si>
+  <si>
+    <t>PF10</t>
+  </si>
+  <si>
+    <t>FMC_INTR, DCMI_D11, LCD_DE, EVENTOUT, ADC3_IN8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -264,22 +511,32 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -302,35 +559,370 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -633,52 +1225,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="124.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="17">
+        <v>57</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>57</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="F2" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="20">
         <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -687,13 +1285,14 @@
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+      <c r="E3" s="15"/>
+      <c r="F3" s="12"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="20">
         <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -702,13 +1301,14 @@
       <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="6"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="E4" s="15"/>
+      <c r="F4" s="12"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="20">
         <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -717,13 +1317,14 @@
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="6"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="E5" s="15"/>
+      <c r="F5" s="12"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="20">
         <v>88</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -732,13 +1333,14 @@
       <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="6"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+      <c r="E6" s="15"/>
+      <c r="F6" s="12"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="20">
         <v>87</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -747,13 +1349,14 @@
       <c r="C7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="6"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+      <c r="E7" s="15"/>
+      <c r="F7" s="12"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="20">
         <v>116</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -762,13 +1365,14 @@
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="6"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+      <c r="E8" s="15"/>
+      <c r="F8" s="12"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="20">
         <v>113</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -777,28 +1381,30 @@
       <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="6"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+      <c r="E9" s="15"/>
+      <c r="F9" s="12"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="20">
         <v>112</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+      <c r="E10" s="15"/>
+      <c r="F10" s="12"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="20">
         <v>111</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -807,13 +1413,14 @@
       <c r="C11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="6"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="E11" s="15"/>
+      <c r="F11" s="12"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="20">
         <v>99</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -822,13 +1429,14 @@
       <c r="C12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+      <c r="E12" s="15"/>
+      <c r="F12" s="12"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="20">
         <v>98</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -837,13 +1445,14 @@
       <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+      <c r="E13" s="15"/>
+      <c r="F13" s="12"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="20">
         <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -852,13 +1461,14 @@
       <c r="C14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E14" s="6"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+      <c r="D14" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="15"/>
+      <c r="F14" s="12"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="20">
         <v>47</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -867,13 +1477,14 @@
       <c r="C15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="6"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="D15" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="15"/>
+      <c r="F15" s="12"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="20">
         <v>133</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -882,96 +1493,186 @@
       <c r="C16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="6"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="D16" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="15"/>
+      <c r="F16" s="12"/>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="23">
         <v>135</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E17" s="6"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="4">
-        <v>10</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="D17" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E17" s="16"/>
+      <c r="F17" s="13"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="17">
+        <v>139</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="D18" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="23">
+        <v>140</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="27"/>
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="32">
+        <v>13</v>
+      </c>
+      <c r="B20" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="12"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="38">
+        <v>22</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="30"/>
+      <c r="F21" s="12"/>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="35">
+        <v>26</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="31"/>
+      <c r="F22" s="12"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="32">
+        <v>124</v>
+      </c>
+      <c r="B23" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="F23" s="12"/>
+    </row>
+    <row r="24" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="35">
+        <v>129</v>
+      </c>
+      <c r="B24" s="36" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>11</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="4">
-        <v>12</v>
-      </c>
-      <c r="B20" s="4" t="s">
+      <c r="C24" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
-        <v>119</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>63</v>
-      </c>
+      <c r="D24" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" s="27"/>
+      <c r="F24" s="13"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="5"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="5"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
     <mergeCell ref="E2:E17"/>
     <mergeCell ref="E18:E19"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F2:F17"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="F18:F24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>